<commit_message>
invalid data removed from
</commit_message>
<xml_diff>
--- a/testData/LoginData.xlsx
+++ b/testData/LoginData.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\playwright\testData\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4E9FD810-7315-4DCF-9676-E8D57679C714}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{043516E0-4BCE-4288-B79B-A600D23B3034}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16" uniqueCount="11">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="9">
   <si>
     <t>username</t>
   </si>
@@ -46,12 +46,6 @@
   </si>
   <si>
     <t>yes</t>
-  </si>
-  <si>
-    <t>locked_out_user</t>
-  </si>
-  <si>
-    <t>error</t>
   </si>
   <si>
     <t>problem_user</t>
@@ -378,7 +372,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D4"/>
+  <dimension ref="A1:D3"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="27.109375" customWidth="1"/>
@@ -408,7 +402,7 @@
         <v>5</v>
       </c>
       <c r="C2" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="D2" s="1" t="s">
         <v>6</v>
@@ -425,20 +419,6 @@
         <v>8</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A4" t="s">
-        <v>9</v>
-      </c>
-      <c r="B4" t="s">
-        <v>5</v>
-      </c>
-      <c r="C4" t="s">
-        <v>10</v>
-      </c>
-      <c r="D4" s="1" t="s">
         <v>6</v>
       </c>
     </row>

</xml_diff>